<commit_message>
ran full submissions tests, updated refernce to generarted files
</commit_message>
<xml_diff>
--- a/submissions_test/assignment_01.xlsx
+++ b/submissions_test/assignment_01.xlsx
@@ -521,17 +521,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Experience the pinnacle of mobile technology with the Apple iPhone 15 Pro. Powered by the groundbreaking A17 Pro chip, this compact powerhouse delivers lightning-fast performance and an incredibly smooth 120Hz ProMotion display.  The durable titanium frame and Ceramic Shield glass ensure lasting protection, while USB-C fast charging keeps you connected without delay. Backed by Apple's one-year limited warranty, the iPhone 15 Pro is your passport to a world of seamless innovation.</t>
+          <t>Experience the power and performance of the Apple iPhone 15 Pro.  This compact powerhouse boasts the blazing-fast A17 Pro chip, a stunning 120Hz ProMotion display for ultra-smooth scrolling, and the convenience of USB-C fast charging. Crafted with a durable titanium frame and protected by Ceramic Shield glass, the iPhone 15 Pro is built to last. Backed by Apple's 1-year limited warranty, you can enjoy peace of mind with your purchase.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1276.4</v>
+        <v>1568.7</v>
       </c>
       <c r="G2" t="n">
         <v>274</v>
       </c>
       <c r="H2" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -565,17 +565,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Capture life's every detail with the stunning 200MP camera on the Samsung Galaxy S24 Ultra. This powerhouse phone boasts a vibrant 120Hz AMOLED display, making every image and video come to life. Plus, the integrated S-Pen opens up a world of creative possibilities right at your fingertips. Crafted with a durable Armor Aluminum frame and scratch-resistant Gorilla Glass Victus, the S24 Ultra is built to last. Backed by a 1-year limited warranty, you can experience the future of mobile technology with confidence.</t>
+          <t>Capture the world in stunning detail with the Samsung Galaxy S24 Ultra. Its revolutionary 200MP camera lets you freeze moments in breathtaking clarity, while the S-Pen unlocks a world of creative possibilities. Experience smooth scrolling and vibrant colors on the 120Hz AMOLED display, housed in a durable Armor Aluminum frame with protective Gorilla Glass Victus.  Rest assured knowing your investment is protected by a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1102.4</v>
+        <v>1058.6</v>
       </c>
       <c r="G3" t="n">
         <v>274</v>
       </c>
       <c r="H3" t="n">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -609,17 +609,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Experience the power and innovation of the Google Pixel 8 Pro. Fueled by the cutting-edge Tensor G3 chip, this smartphone delivers exceptional performance for all your tasks. Capture stunning photos with the 50MP camera, enhanced by Google's Magic Eraser for effortless editing.  The sleek design boasts a durable matte glass back and aluminum frame, offering both style and protection. Backed by a 1-year limited warranty, the Pixel 8 Pro is ready to elevate your mobile experience.</t>
+          <t>Experience the pinnacle of mobile innovation with the Google Pixel 8 Pro. Powered by the lightning-fast Tensor G3 chip, this smartphone seamlessly handles demanding tasks and captures stunning photos with its 50MP camera.  Magic Eraser allows you to effortlessly remove unwanted objects from your images, making every shot perfect. The sleek matte glass back and durable aluminum frame  ensure both style and longevity. Backed by a 1-year limited warranty, the Pixel 8 Pro is an investment in premium mobile excellence.</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2171.1</v>
+        <v>1264.9</v>
       </c>
       <c r="G4" t="n">
         <v>271</v>
       </c>
       <c r="H4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -653,17 +653,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Escape into your own world of sound with the Sony WH-1000XM5 Headphones.  Experience unparalleled audio bliss thanks to advanced active noise cancelling technology, silencing the world around you. Enjoy up to 30 hours of playtime on a single charge, perfect for long commutes or flights.  These comfortable headphones feature plush synthetic leather earcups, ensuring a cozy fit for extended listening sessions. Backed by a 1-year limited warranty, the Sony WH-1000XM5 Headphones deliver exceptional audio quality and reliability.</t>
+          <t>Escape into a world of pure sound with the Sony WH-1000XM5 Headphones.  Experience exceptional noise cancellation, allowing you to focus on your music, podcasts, or work without distractions.  Enjoy up to 30 hours of battery life on a single charge, and seamlessly connect to your devices with the latest Bluetooth 5.2 technology.  The generously sized, synthetic leather earcups provide a comfortable fit for extended listening sessions. Backed by a 1-year limited warranty, these headphones are a smart investment in your audio enjoyment.</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1699.2</v>
+        <v>3056</v>
       </c>
       <c r="G5" t="n">
         <v>271</v>
       </c>
       <c r="H5" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -697,17 +697,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Experience audio nirvana with the Bose QuietComfort Ultra Earbuds.  These award-winning earbuds deliver a personalized sound experience thanks to CustomTune sound calibration, while Active Noise Cancellation ensures you can focus on your music, not the world around you.  The IPX4 water resistance rating makes them perfect for workouts, and the comfortable silicone ear tips provide a secure, all-day fit. Backed by a 1-year limited warranty, the QuietComfort Ultra Earbuds are your ticket to premium audio bliss.</t>
+          <t>Experience unparalleled audio bliss with the Bose QuietComfort Ultra Earbuds.  These award-winning earbuds boast CustomTune sound calibration, ensuring a personalized listening experience tailored to your ears.  Advanced Active Noise Cancellation (ANC) technology silences the world around you, allowing you to fully immerse yourself in your music.  With an IPX4 rating, they're ready for your active lifestyle, and the comfortable silicone ear tips provide a secure and snug fit.  Backed by a 1-year limited warranty, you can enjoy your audio sanctuary with confidence.</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2213.9</v>
+        <v>1554.9</v>
       </c>
       <c r="G6" t="n">
         <v>260</v>
       </c>
       <c r="H6" t="n">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -741,17 +741,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The Amazon Echo Dot (5th Gen) is your smart home's perfect companion. This compact device packs a punch with its improved bass, making it ideal for enjoying music throughout your home.  Control your smart devices, get answers to questions, and check the weather, all with the power of Alexa. Plus, with its temperature sensor, the Echo Dot can even help you keep your home comfortable. Crafted from sustainably sourced recycled fabric mesh, the Echo Dot (5th Gen) is good for both your home and the planet. Backed by a 1-year limited warranty, you can enjoy peace of mind with your purchase.</t>
+          <t>Bring Alexa's smarts and a touch of eco-consciousness to your home with the Amazon Echo Dot (5th Gen). This compact device boasts an improved bass for richer sound, while the built-in temperature sensor adds a convenient layer of home monitoring. Powered by the Alexa voice assistant, it's your gateway to music, information, and hands-free control. Wrapped in sustainably sourced, recycled fabric mesh, the Echo Dot (5th Gen) is a smart choice for both your lifestyle and the planet. Enjoy peace of mind with a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1099.5</v>
+        <v>1546.9</v>
       </c>
       <c r="G7" t="n">
         <v>260</v>
       </c>
       <c r="H7" t="n">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -785,17 +785,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The Dell XPS 13 9310 Laptop is the perfect blend of power and portability. Its sleek CNC aluminum and carbon-fiber palmrest design not only looks stunning but also feels incredibly durable. With a vibrant 13.4″ FHD+ display, you'll enjoy crystal-clear visuals for all your work and entertainment. Powered by an Intel Core i5 processor and equipped with the lightning-fast Thunderbolt 4, this compact laptop handles demanding tasks with ease.  Rest assured with Dell's 1-year limited hardware warranty.</t>
+          <t>The Dell XPS 13 9310 Laptop is the perfect blend of power and portability. Its stunning 13.4″ FHD+ display brings your content to life, while the Intel Core i5 processor ensures smooth performance for all your tasks.  With Thunderbolt 4 connectivity and a compact design, you can stay productive on the go.  Crafted from premium CNC aluminum and a comfortable carbon-fiber palmrest, this laptop not only looks great but feels even better. Your XPS 13 9310 is backed by a 1-year limited hardware warranty for peace of mind.</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>982.4</v>
+        <v>1436.7</v>
       </c>
       <c r="G8" t="n">
         <v>280</v>
       </c>
       <c r="H8" t="n">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -829,17 +829,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The Apple MacBook Air 13″ (M3) is a powerful and portable masterpiece designed for the modern professional. Driven by the innovative M3 chip, this Air delivers exceptional performance while remaining incredibly energy efficient. With an impressive 18-hour battery life and a crystal-clear 1080p camera, you'll stay productive and connected all day long. Crafted from a durable, recycled aluminum unibody, the MacBook Air 13″ (M3) is a testament to both style and sustainability. Backed by a 1-year limited warranty, you can experience peace of mind with every use.</t>
+          <t>The Apple MacBook Air 13″ (M3) is a powerful and portable laptop designed for everyday productivity and entertainment. Powered by the innovative M3 chip, it delivers exceptional performance while being incredibly energy efficient, offering up to 18 hours of battery life.  Enjoy crystal-clear video calls with the 1080p camera, and experience the sleek and durable design of the recycled aluminum unibody. Backed by a 1-year limited warranty, the MacBook Air (M3) is the perfect companion for work, school, or leisure.</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1708.6</v>
+        <v>1303.1</v>
       </c>
       <c r="G9" t="n">
         <v>274</v>
       </c>
       <c r="H9" t="n">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -873,18 +873,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The Microsoft Surface Pro 10 is the perfect blend of power and portability. 
-Equipped with an Intel Core Ultra processor, this compact powerhouse handles demanding tasks with ease. The detachable keyboard allows you to seamlessly switch between laptop and tablet modes, while the stunning 13″ PixelSense display brings your content to life.  Crafted from a durable magnesium alloy chassis, the Surface Pro 10 is built to last, backed by a 1-year limited warranty for your peace of mind.</t>
+          <t>The Microsoft Surface Pro 10 is the perfect blend of power and portability. Equipped with an Intel Core Ultra processor, this compact tablet seamlessly transitions from work to play. Its stunning 13” PixelSense display and detachable keyboard offer a versatile experience, while the lightweight magnesium alloy chassis ensures effortless mobility.  Enjoy peace of mind with Microsoft's 1-year limited warranty, covering any defects in materials or workmanship.</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1124.8</v>
+        <v>986.9</v>
       </c>
       <c r="G10" t="n">
         <v>263</v>
       </c>
       <c r="H10" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -918,17 +917,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The Garmin Forerunner 255 is the perfect running companion for athletes of all levels. Its multi-band GPS ensures accurate tracking, while HRV status provides insights into your recovery.  Enjoy up to 14 days of battery life, so you can focus on your runs, not charging.  Built with durable fiber-reinforced polymer, this watch is ready for anything. Backed by a 1-year limited warranty, you can be confident in your investment.</t>
+          <t>The Garmin Forerunner 255 is the perfect running companion for serious athletes and casual joggers alike.  With multi-band GPS for precise tracking and HRV status to monitor your recovery, you'll gain valuable insights into your performance. The long-lasting 14-day battery means you can go the distance without worry.  Crafted from durable fiber-reinforced polymer, the Forerunner 255 is built to withstand the demands of your training. Backed by a 1-year limited warranty, you can purchase with confidence.</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1166.1</v>
+        <v>1560.6</v>
       </c>
       <c r="G11" t="n">
         <v>272</v>
       </c>
       <c r="H11" t="n">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -962,11 +961,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>The Fitbit Charge 6 is the perfect fitness companion, designed to help you reach your health goals with ease.  Featuring a sleek aluminum case and available in a variety of colors to match your style, this wearable tracks your heart rate and provides built-in GPS for accurate distance and pace information.  Enjoy up to 7 days of battery life between charges, so you can stay connected and motivated throughout your week.  Backed by a 1-year limited warranty, the Charge 6 is a reliable and stylish choice for any fitness enthusiast.</t>
+          <t>Stay on top of your fitness goals with the stylish and functional Fitbit Charge 6.  This sleek aluminum case tracker boasts a built-in GPS to map your runs and a heart-rate monitor to track your progress.  Enjoy up to 7 days of battery life, so you can wear it day and night without worry. With multiple color options to choose from, you're sure to find the perfect Charge 6 to match your personal style. Backed by a 1-year limited warranty, you can experience fitness tracking with confidence.</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1032.2</v>
+        <v>1324</v>
       </c>
       <c r="G12" t="n">
         <v>263</v>
@@ -1006,17 +1005,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Capture life's most epic moments in stunning detail with the GoPro HERO12 Black. This rugged powerhouse shoots incredible 5.3K60 video, stabilized by the advanced HyperSmooth 6.0 technology. Dive right in, thanks to its waterproof design that can handle depths of up to 10 meters. Plus, the large capacity ensures you'll never miss a beat. Built tough with durable polycarbonate, the HERO12 Black is ready for any adventure. Backed by a 1-year limited warranty, you can explore with confidence.</t>
+          <t>Capture every epic moment in stunning detail with the GoPro HERO12 Black.  This rugged powerhouse shoots incredible 5.3K60 video, stabilized by the advanced HyperSmooth 6.0 technology, ensuring your footage is always smooth and cinematic. Built to withstand the elements with a durable polycarbonate shell, the HERO12 Black is waterproof to 10m, ready for any adventure.  And with its large capacity, you can record all the action without worrying about running out of space. Backed by a 1-year limited warranty, the HERO12 Black is your ultimate tool for capturing life's greatest moments.</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1095.1</v>
+        <v>1407.6</v>
       </c>
       <c r="G13" t="n">
         <v>270</v>
       </c>
       <c r="H13" t="n">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1050,17 +1049,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Capture stunning 4K/60fps footage with the DJI Mini 4 Pro, a lightweight drone that's perfect for cinematic adventures. Weighing in at under 250 g, it's incredibly portable while still boasting omnidirectional obstacle sensing for safe and effortless flights.  Crafted from durable composite plastic, the Mini 4 Pro is built to withstand the rigors of exploration. Backed by a 1-year limited warranty, you can fly with confidence knowing your investment is protected.</t>
+          <t>Capture stunning 4K footage at 60fps with the DJI Mini 4 Pro drone.  Weighing in at under 250 grams, this nimble drone is perfect for capturing breathtaking aerial shots.  Omnidirectional obstacle sensing keeps you safe while flying, and with a 4.7/5 star rating, you can be confident you're getting a high-quality product.  Crafted from durable composite plastic, the Mini 4 Pro is built to last, backed by a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1146.4</v>
+        <v>2483.5</v>
       </c>
       <c r="G14" t="n">
         <v>274</v>
       </c>
       <c r="H14" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1094,17 +1093,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Experience gaming like never before with the Nintendo Switch OLED. Its vibrant 7″ OLED screen brings your favorite games to life with stunning clarity and rich colors, whether you're playing in handheld or docked mode.  With 64GB of storage, you'll have plenty of space for your game library.  The sleek plastic chassis is both durable and comfortable to hold, making it perfect for on-the-go gaming.  Backed by a 1-year limited warranty, the Switch OLED is ready to provide endless hours of entertainment.</t>
+          <t>Experience immersive gaming like never before with the Nintendo Switch OLED. Its vibrant 7-inch OLED screen brings your games to life with stunning colors and deep blacks, whether you're playing in docked or handheld mode.  With 64GB of storage, there's plenty of space for all your favorite titles.  Crafted with a durable plastic chassis, the Switch OLED is ready for hours of entertainment.  Enjoy peace of mind with our 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>989.6</v>
+        <v>1045.8</v>
       </c>
       <c r="G15" t="n">
         <v>263</v>
       </c>
       <c r="H15" t="n">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1138,17 +1137,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Experience the future of gaming with the PlayStation 5 Slim.  Immerse yourself in stunning visuals with ray tracing technology and feel every detail with the innovative haptic feedback controller.  The 1TB SSD ensures lightning-fast loading times, while the long-lasting battery keeps you playing for hours.  Crafted with a sleek plastic shell, this console is a stylish addition to any entertainment setup. Your purchase is protected by a 1-year limited warranty, giving you peace of mind for your gaming adventures.</t>
+          <t>Experience the future of gaming with the PlayStation 5 Slim. This sleek console, crafted with a durable plastic shell, delivers breathtaking visuals thanks to its advanced ray tracing technology. Feel every jolt and nuance with the innovative haptic feedback controller, and enjoy lightning-fast load times with the spacious 1TB SSD.  The PlayStation 5 Slim offers long-lasting battery life, ensuring your gaming sessions last as long as your desire. Backed by a 1-year limited warranty, you can dive into immersive worlds with confidence.</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1028.5</v>
+        <v>1104</v>
       </c>
       <c r="G16" t="n">
         <v>262</v>
       </c>
       <c r="H16" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1182,17 +1181,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Experience next-gen gaming with the Xbox Series X. This powerhouse console boasts a 12 TFLOPS GPU and a blazing-fast 1 TB SSD, delivering breathtaking 4K visuals at up to 120Hz for incredibly smooth gameplay. The sleek matte black casing complements any gaming setup, while the long-lasting battery ensures hours of uninterrupted fun. Backed by a 1-year limited warranty, the Xbox Series X is ready to elevate your gaming experience to new heights.</t>
+          <t>Experience the pinnacle of gaming performance with the Xbox Series X.  This powerhouse console boasts a stunning 12 teraflop GPU and a lightning-fast 1TB SSD, delivering breathtaking 4K visuals at up to 120Hz. Immerse yourself in a world of seamless gameplay and vibrant colors thanks to its matte black casing.  Enjoy long-lasting battery life and the peace of mind that comes with a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2367.9</v>
+        <v>1188.8</v>
       </c>
       <c r="G17" t="n">
         <v>274</v>
       </c>
       <c r="H17" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1226,17 +1225,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>The Instant Pot Duo 6-Quart is your kitchen's new secret weapon! This versatile 7-in-1 multicooker lets you pressure cook, slow cook, sauté, steam, make rice, and more, all in one convenient appliance. Crafted with durable 18/8 stainless steel, including the inner pot, it's built to last.  At a light weight, it's easy to maneuver, and with a powerful 1000W heating element, you'll be enjoying delicious meals in no time. Backed by a 1-year limited warranty, the Instant Pot Duo 6-Quart is the perfect choice for busy cooks who want it all.</t>
+          <t>The Instant Pot Duo 6-Quart is a versatile kitchen essential, acting as a pressure cooker, slow cooker, rice cooker, steamer, sauté pan, yogurt maker, and warmer—all in one!  Its 18/8 stainless steel inner pot is both durable and easy to clean, while the 1000W heating element ensures quick and efficient cooking. Its lightweight design makes it easy to maneuver around your kitchen, and with a 1-year limited warranty, you can be confident in your purchase.</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1254.9</v>
+        <v>1222.2</v>
       </c>
       <c r="G18" t="n">
         <v>279</v>
       </c>
       <c r="H18" t="n">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1270,17 +1269,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Elevate your coffee experience with the Keurig K-Supreme Plus Smart. This sophisticated machine boasts multistream extraction technology for a perfectly balanced brew every time, along with BrewID intelligence that recognizes and optimizes each K-Cup pod.  With a spacious 78-ounce reservoir, you'll enjoy fewer refills and more time savoring your favorite flavors. The sleek design, featuring brushed stainless steel accents, complements any kitchen. Backed by a 1-year limited warranty, the K-Supreme Plus Smart is the smart choice for coffee lovers.</t>
+          <t>Upgrade your coffee routine with the Keurig K-Supreme Plus Smart. This smart brewer boasts a large 78oz reservoir, eliminating frequent refills, and features multistream extraction technology for a perfectly brewed cup every time.  BrewID technology even recognizes your K-Cup pod, optimizing brewing parameters for the ultimate flavor.  Crafted with sleek brushed stainless steel accents, the K-Supreme Plus Smart is both stylish and functional, backed by a 1-year limited warranty for worry-free brewing.</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>997.9</v>
+        <v>1066.1</v>
       </c>
       <c r="G19" t="n">
         <v>265</v>
       </c>
       <c r="H19" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1314,17 +1313,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The Vitamix 5200 Blender is a powerful and versatile kitchen essential. With its 2-hp motor and variable speed control, you can effortlessly blend smoothies, soups, sauces, and more to perfection.  The self-cleaning function makes cleanup a breeze, while the BPA-free Tritan jar ensures your ingredients are always safe. Backed by a 7-year warranty, the Vitamix 5200 is a reliable investment for years of delicious homemade creations.</t>
+          <t>The Vitamix 5200 Blender is a powerhouse in your kitchen, ready to blend anything from smoothies to soups with ease. Its powerful 2-hp motor and variable speed settings give you complete control, while the self-cleaning function makes cleanup a breeze. Crafted from a BPA-free Tritan jar, this blender is built to last and is backed by a  7-year warranty for your peace of mind.  Make healthy and delicious meals effortlessly with the Vitamix 5200.</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>851.9</v>
+        <v>1270</v>
       </c>
       <c r="G20" t="n">
         <v>266</v>
       </c>
       <c r="H20" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1358,17 +1357,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tired of hidden dust? The Dyson V15 Detect revolutionizes cleaning with its groundbreaking laser dust detection, illuminating even the tiniest particles.  Enjoy powerful suction and a remarkable 60-minute runtime, all while benefiting from HEPA filtration that traps allergens and pollutants. This sleek vacuum, crafted from durable polycarbonate and aluminum, is not only efficient but also built to last. Backed by a 2-year warranty, the Dyson V15 Detect is your key to a truly clean and healthy home.</t>
+          <t>Experience the ultimate clean with the Dyson V15 Detect Vacuum. This powerful cordless vacuum utilizes advanced laser dust detection to reveal hidden dirt you never knew existed. With HEPA filtration, you can breathe easy knowing allergens and fine particles are captured, leaving your home truly spotless. Enjoy up to 60 minutes of run time on a single charge, making tackling any mess a breeze.  Crafted from durable polycarbonate and aluminum, the V15 Detect is built to last, backed by a 2-year parts and labor warranty for your peace of mind.</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>874.2</v>
+        <v>1348.2</v>
       </c>
       <c r="G21" t="n">
         <v>265</v>
       </c>
       <c r="H21" t="n">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1402,17 +1401,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Meet the iRobot Roomba j7+, an award-winning robot vacuum designed to revolutionize your cleaning routine.  Equipped with PrecisionVision navigation, it expertly maps and navigates your home, avoiding obstacles with ease.  The self-emptying Clean Base ensures uninterrupted cleaning for weeks, while seamless Alexa integration lets you control it with your voice.  Housed in durable plastic, the Roomba j7+ is backed by a 1-year limited warranty, giving you peace of mind.</t>
+          <t>Meet the iRobot Roomba j7+, a robotic vacuum that combines award-winning design with intelligent navigation.  Equipped with PrecisionVision, it expertly maps your home and avoids obstacles, leaving no corner untouched.  The self-emptying Clean Base ensures weeks of mess-free operation, while compatibility with Alexa lets you control it with your voice.  Crafted with durable plastic housing, the j7+ is backed by a 1-year limited warranty, giving you peace of mind.</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>906.9</v>
+        <v>1225.1</v>
       </c>
       <c r="G22" t="n">
         <v>263</v>
       </c>
       <c r="H22" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1446,17 +1445,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>The Yeti Rambler 20oz Tumbler is your perfect companion for conquering any adventure. Crafted from durable kitchen-grade stainless steel, this compact tumbler boasts double-wall vacuum insulation to keep your drinks icy cold or steaming hot for hours on end.  The MagSlider lid ensures a secure seal, while its convenient size fits perfectly in your hand or cup holder. Backed by Yeti's legendary 5-year warranty, the Rambler is built to last.</t>
+          <t>Keep your drinks perfectly chilled or steaming hot for hours on end with the Yeti Rambler 20 oz Tumbler. Crafted from durable, kitchen-grade stainless steel, this compact tumbler boasts double-wall vacuum insulation to prevent temperature loss and condensation. The convenient MagSlider lid ensures a secure seal and easy sipping, making it perfect for on-the-go adventures. Backed by Yeti's legendary 5-year warranty, the Rambler is built to last and is a worthy investment for any beverage enthusiast.</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>860.8</v>
+        <v>1272.5</v>
       </c>
       <c r="G23" t="n">
         <v>264</v>
       </c>
       <c r="H23" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1490,17 +1489,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>The Stanley Quencher H2.0 40 oz is your ultimate hydration companion.  Crafted from durable, recycled stainless steel, this tumbler keeps your drinks ice cold for hours thanks to its vacuum insulation.  The innovative flow-state lid offers a convenient, spill-proof drinking experience, while the cup-holder friendly design makes it perfect for on-the-go.  And with a long-lasting battery, you can enjoy your perfectly chilled beverages wherever your adventures take you.  Backed by a lifetime warranty, the Stanley Quencher is an investment in lasting refreshment.</t>
+          <t>Stay refreshed all day long with the Stanley Quencher H2.0 40 oz! This durable, vacuum-insulated tumbler is crafted from recycled stainless steel, keeping your drinks icy cold or piping hot for hours.  The innovative flow-state lid lets you sip effortlessly, and its cup-holder friendly design ensures you can take it on the go.  Plus, with a long-lasting battery and a lifetime warranty, you can be confident in your investment.</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1383.1</v>
+        <v>1111.2</v>
       </c>
       <c r="G24" t="n">
         <v>267</v>
       </c>
       <c r="H24" t="n">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1534,17 +1533,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>The Hydro Flask 32 oz Wide Mouth is your perfect companion for all adventures.  Crafted from durable, pro-grade stainless steel and featuring TempShield insulation, this bottle keeps your drinks icy cold or piping hot for hours on end.  The Color Last powder coat ensures your flask stays vibrant no matter how many miles you log.  Compact and convenient, this wide mouth design makes it easy to add ice and clean. Backed by a lifetime warranty, your Hydro Flask is an investment in lasting quality and refreshment.</t>
+          <t>Stay refreshed all day long with the Hydro Flask 32oz Wide Mouth. This compact tumbler is crafted from durable pro-grade stainless steel and features TempShield insulation to keep your drinks ice cold or piping hot for hours.  The Color Last powder coat ensures your Hydro Flask stays looking its best, while the lifetime warranty guarantees its performance.</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1109.4</v>
+        <v>1029.4</v>
       </c>
       <c r="G25" t="n">
         <v>259</v>
       </c>
       <c r="H25" t="n">
-        <v>110</v>
+        <v>73</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1578,17 +1577,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>The Contigo Autoseal West Loop is your perfect on-the-go companion. Crafted from durable stainless steel, this 16-ounce tumbler keeps your drinks hot or cold for hours thanks to its double-wall insulation.  The innovative Autoseal lid ensures worry-free sipping with its spill-proof design, making it ideal for hectic commutes or busy days.  Plus, with Contigo's lifetime warranty, you can enjoy peace of mind knowing your investment is protected.</t>
+          <t>The Contigo Autoseal West Loop is your perfect companion for busy days.  This 16-ounce stainless steel tumbler keeps your drinks hot or cold for hours with its double-wall insulation, while the autoseal spill-proof lid ensures worry-free sipping on the go. Its compact design fits easily in your bag, making it ideal for commuting, workouts, or simply running errands. Plus, with Contigo's lifetime warranty, you can enjoy this reliable tumbler for years to come.</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>836.9</v>
+        <v>1235.2</v>
       </c>
       <c r="G26" t="n">
         <v>261</v>
       </c>
       <c r="H26" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1622,17 +1621,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Experience the perfect blend of responsiveness and comfort with the Nike Air Zoom Pegasus 40.  Engineered with innovative React foam and Zoom Air units, these shoes deliver a smooth, energy-efficient ride for every stride. The breathable engineered mesh upper keeps your feet feeling cool and supported, mile after mile. Backed by a 2-year manufacturer warranty, the Pegasus 40 is built to be your trusted running companion.</t>
+          <t>Experience effortless strides with the Nike Air Zoom Pegasus 40. This versatile running shoe combines the responsiveness of Zoom Air units with the plush cushioning of React foam, delivering energy-efficient performance mile after mile. The breathable engineered mesh upper keeps your feet comfortable and supported, whether you're tackling daily runs or pushing your limits. Backed by a 2-year manufacturer warranty, the Pegasus 40 is a reliable companion for your running journey.</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>779</v>
+        <v>1082.2</v>
       </c>
       <c r="G27" t="n">
         <v>260</v>
       </c>
       <c r="H27" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1666,17 +1665,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Experience the ultimate in lightweight comfort with the Adidas Ultraboost Light. These running shoes boast a responsive Light BOOST midsole for a springy feel with every stride, while the breathable Primeknit+ upper provides a snug, supportive fit.  Grippy Continental rubber ensures superior traction on a variety of surfaces. Backed by a 2-year manufacturer warranty, the Ultraboost Light is ready to elevate your running experience.</t>
+          <t>Experience the ultimate in lightweight comfort with the Adidas Ultraboost Light. Its innovative Light BOOST midsole delivers responsive cushioning, while the Primeknit+ upper provides a breathable, supportive fit.  Grippy Continental rubber ensures excellent traction on any surface. Backed by a 2-year manufacturer warranty, these shoes are built for long-lasting performance and satisfaction.  Rated 4.7 out of 5 stars, the Adidas Ultraboost Light is a top choice for runners and everyday wear.</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>850.4</v>
+        <v>1144.1</v>
       </c>
       <c r="G28" t="n">
         <v>266</v>
       </c>
       <c r="H28" t="n">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -1710,17 +1709,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Stay warm and comfortable in all conditions with the North Face ThermoBall Eco Jacket. This compact jacket is filled with synthetic ThermoBall insulation, providing exceptional warmth without the bulk. The DWR finish helps repel water and snow, keeping you dry and protected. Crafted from 100% recycled nylon, this jacket is both durable and environmentally friendly. Backed by The North Face's lifetime warranty, you can trust that this jacket will be a reliable companion for years to come.</t>
+          <t>Stay warm and comfortable in any weather with The North Face ThermoBall Eco Jacket.  This jacket is packed with synthetic ThermoBall insulation that mimics the warmth of down, keeping you cozy even when wet.  The DWR finish sheds light rain and snow, while the compact design makes it easy to pack for any adventure. Made from 100% recycled nylon, this jacket is as good for the planet as it is for you, and it's backed by The North Face's lifetime warranty for ultimate peace of mind.</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>938.6</v>
+        <v>1261.2</v>
       </c>
       <c r="G29" t="n">
         <v>259</v>
       </c>
       <c r="H29" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -1754,17 +1753,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>The Patagonia Black Hole 32L Backpack is built for adventure, no matter the weather. Crafted from durable, 100% recycled polyester ripstop, this large-capacity pack keeps your gear safe and dry.  A padded laptop sleeve and comfortable straps ensure you can carry everything you need with ease.  Backed by Patagonia's lifetime warranty, the Black Hole 32L is an investment in quality and performance that will last for years to come.</t>
+          <t>The Patagonia Black Hole 32L Backpack is built for adventure with a large capacity to carry all your essentials. Made from durable, 100% recycled polyester ripstop, this weather-resistant backpack is ready for anything.  A padded laptop sleeve protects your devices, and the comfortable, padded straps ensure a comfortable carry even when fully loaded. Backed by Patagonia's legendary lifetime warranty, the Black Hole 32L is an investment in quality and performance that will last for years to come.</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>825.5</v>
+        <v>1591.5</v>
       </c>
       <c r="G30" t="n">
         <v>264</v>
       </c>
       <c r="H30" t="n">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -1798,17 +1797,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>The Osprey Farpoint 40 is the perfect travel companion, designed for both comfort and efficiency.  This carry-on sized backpack boasts a stowaway harness, perfect for navigating bustling airports or exploring cobblestone streets.  Keep your laptop safe and secure in the dedicated laptop sleeve, while the durable 450D recycled nylon construction ensures this bag can handle the rigors of your adventures. And with Osprey's legendary lifetime warranty, you can travel with confidence knowing your Farpoint 40 is built to last.</t>
+          <t>The Osprey Farpoint 40 is the perfect travel companion, blending functionality and sustainability. Its carry-on size ensures hassle-free air travel, while the stowaway harness allows for effortless transitions between backpack and shoulder bag.  Keep your essentials organized with the dedicated laptop sleeve. Crafted from durable, energy-efficient 450D recycled nylon, the Farpoint 40 is built to last, backed by Osprey's legendary lifetime warranty.</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>931</v>
+        <v>1384.6</v>
       </c>
       <c r="G31" t="n">
         <v>261</v>
       </c>
       <c r="H31" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -1842,17 +1841,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Embark on an epic build with the LEGO Star Wars Millennium Falcon 75192. This incredible set boasts 7,541 pieces, allowing you to meticulously recreate the iconic ship's intricate details, from its bustling interior to its legendary exterior.  With a comprehensive collection of minifigs included, you'll be ready to stage thrilling adventures straight from the Star Wars galaxy. Constructed from durable ABS plastic bricks and backed by a lifetime warranty for missing pieces, this set is built to last, ensuring countless hours of creative play and display.</t>
+          <t>Calling all Star Wars fans and LEGO builders! The Millennium Falcon 75192 is the ultimate build, boasting a staggering 7,541 pieces and incredible detail both inside and out.  With iconic minifigures included, you can recreate your favorite scenes from the films. Constructed from durable ABS plastic bricks, this set is built to last. Plus, with LEGO's lifetime guarantee for missing bricks, you can rest assured your Falcon will always be in top shape.</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1111.8</v>
+        <v>1312.2</v>
       </c>
       <c r="G32" t="n">
         <v>270</v>
       </c>
       <c r="H32" t="n">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
@@ -1886,17 +1885,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bring a touch of nature's beauty indoors with the LEGO Icons Botanical Orchid 10311. This stunning build features 608 pieces, allowing you to create a lifelike orchid with adjustable blooms for a personalized touch. Crafted from high-quality ABS plastic bricks, this decorative set is sure to be a conversation starter. Plus, enjoy peace of mind with LEGO's lifetime guarantee, ensuring you can always replace any missing bricks.</t>
+          <t>Bring the beauty of nature indoors with the LEGO Icons Botanical Orchid 10311. This stunning 608-piece set lets you create a realistic orchid display with adjustable blooms for a personalized touch.  Crafted from durable ABS plastic bricks, the orchid is a decorative masterpiece for any home. Plus, with LEGO's lifetime guarantee, you can be sure that any missing bricks will be replaced, ensuring your orchid blossoms forever.</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>811.9</v>
+        <v>1126.8</v>
       </c>
       <c r="G33" t="n">
         <v>265</v>
       </c>
       <c r="H33" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -1930,17 +1929,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Escape into a world of endless reading with the Kindle Paperwhite 11th Gen. Its spacious 6.8” glare-free display makes reading a joy, whether you're curled up indoors or soaking up the sun.  With a remarkable 10-week battery life, you can savor countless stories without interruption.  The compact design and USB-C charging add to its convenience.  Crafted with sustainable recycled plastic, the Kindle Paperwhite 11th Gen is as good for the planet as it is for your reading pleasure, backed by a 1-year limited warranty.</t>
+          <t>Escape to endless reading adventures with the Kindle Paperwhite 11th Gen. Its expansive 6.8″ glare‑free display brings your favorite books to life, while the 10‑week battery ensures you're never left wanting.  This compact device, crafted with recycled plastic, is perfect for taking your literary escapism wherever you go. Plus, with a 1‑year limited warranty, you can read with confidence.</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1076.5</v>
+        <v>1111.7</v>
       </c>
       <c r="G34" t="n">
         <v>271</v>
       </c>
       <c r="H34" t="n">
-        <v>127</v>
+        <v>94</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -1974,17 +1973,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>The Kobo Libra 2 is your perfect reading companion, wherever your adventures take you. This lightweight eReader boasts a gorgeous 7″ E Ink Carta display, delivering crisp text and a paper-like reading experience.  Dive into your favorite books, even by the pool, thanks to its IPX8 waterproof rating.  Enjoy audiobooks wirelessly with Bluetooth connectivity and get lost in your next great story. Backed by a 1-year limited warranty, the Kobo Libra 2 is built to last and enhance your reading journey.</t>
+          <t>Dive into your next adventure with the Kobo Libra 2. This lightweight e-reader boasts a beautiful 7″ E Ink Carta display, perfect for hours of comfortable reading. Enjoy audiobooks wirelessly via Bluetooth and don't worry about splashes thanks to its IPX8 waterproof rating.  Crafted with a durable plastic chassis, the Libra 2 is built to keep up with your busy life, backed by a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>968</v>
+        <v>1104.2</v>
       </c>
       <c r="G35" t="n">
         <v>262</v>
       </c>
       <c r="H35" t="n">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
@@ -2018,17 +2017,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>The Anker Soundcore Motion+ speaker delivers a powerful 30W audio experience with stunning Hi-Res sound quality. Enjoy your music anywhere, worry-free, thanks to its IPX7 waterproof rating and durable aluminum grille.  The Motion+ is designed to be energy efficient, so you can immerse yourself in your favorite tunes for longer. Backed by an 18-month warranty, the Motion+ is a reliable choice for exceptional audio on the go.</t>
+          <t>The Anker Soundcore Motion+ speaker delivers incredible 30W audio with Hi-Res clarity, perfect for immersing yourself in your favorite music.  Its rugged aluminum grille and IPX7 waterproof rating make it ready for any adventure, from poolside parties to hiking trails. Enjoy powerful sound with the peace of mind that comes with Anker's 18-month warranty.</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1931</v>
+        <v>875</v>
       </c>
       <c r="G36" t="n">
         <v>262</v>
       </c>
       <c r="H36" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -2062,17 +2061,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>The Sonos Move 2 brings your favorite music anywhere, anytime. Stream wirelessly via WiFi or Bluetooth with a 24-hour battery life for all-day listening. Automatic Trueplay ensures perfect sound wherever you go, adjusting to your unique environment.  Crafted with a durable, shock-resistant shell, the Move 2 is built to keep up with your adventures. Enjoy peace of mind with a 1-year limited warranty.</t>
+          <t>Take your music anywhere with the Sonos Move 2. This portable speaker delivers rich, powerful sound powered by WiFi and Bluetooth. Enjoy up to 24 hours of playtime on a single charge, and let Trueplay technology automatically optimize sound for your environment. The Move 2's durable, shock-resistant shell is built to withstand your adventures, while the 4.7/5 star rating speaks for itself. Backed by a 1-year limited warranty, the Move 2 is your perfect companion for any occasion.</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>960.4</v>
+        <v>1285.9</v>
       </c>
       <c r="G37" t="n">
         <v>268</v>
       </c>
       <c r="H37" t="n">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -2106,17 +2105,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Unleash a world of color and ambiance in your home with the limited-edition Philips Hue White &amp; Color Ambiance Starter Kit. This innovative kit features 16 million vibrant colors, allowing you to set the perfect mood for any occasion.  Control your lights effortlessly with Bluetooth and Zigbee connectivity, or use your voice with compatible assistants.  Experience the magic of smart lighting with the Philips Hue Starter Kit, backed by a 2-year limited warranty.</t>
+          <t>Unleash a world of color and ambiance with the Philips Hue White &amp; Color Ambiance Starter Kit. This limited-edition set features three plastic bulbs, each capable of illuminating your space in 16 million vibrant hues.  Control your lights effortlessly with Bluetooth or Zigbee connectivity, and even use your voice with compatible assistants.  Add a touch of magic to your home with the Philips Hue starter kit, backed by a 2-year limited warranty for peace of mind.</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>857.8</v>
+        <v>1117</v>
       </c>
       <c r="G38" t="n">
         <v>265</v>
       </c>
       <c r="H38" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -2150,17 +2149,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Enjoy seamless, lightning-fast WiFi throughout your entire home with the TP-Link Deco XE75 Mesh WiFi 6E system. This powerful 3-pack delivers tri-band AXE5400 speeds, conquering even the largest spaces up to 7,200 square feet.  Experience smooth streaming, lag-free gaming, and effortless connectivity for all your devices.  Backed by a 2-year limited warranty, the Deco XE75 offers reliable performance and long-lasting battery life, making it the perfect solution for a truly connected home.</t>
+          <t>Experience seamless, lightning-fast WiFi throughout your entire home with the TP-Link Deco XE75 Mesh WiFi 6E system. This tri-band AXE5400 powerhouse, delivered in a convenient 3-pack, blankets up to 7,200 square feet with reliable coverage. Enjoy long-lasting battery life and peace of mind with a 2-year limited warranty. Upgrade your WiFi experience today with the Deco XE75.</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1028.4</v>
+        <v>1396.1</v>
       </c>
       <c r="G39" t="n">
         <v>281</v>
       </c>
       <c r="H39" t="n">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -2194,17 +2193,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>See and hear everything happening at your doorstep with the Eufy Video Doorbell Dual.  This innovative doorbell boasts dual cameras, giving you a complete view of your porch and detecting packages with precision. Enjoy crystal-clear 2K resolution footage, and rest easy knowing the long-lasting battery keeps it powered up and ready.  Encased in durable plastic, the Eufy Video Doorbell Dual is backed by a 1-year limited warranty for your peace of mind.</t>
+          <t>Experience peace of mind with the Eufy Video Doorbell Dual. This innovative doorbell features dual cameras, capturing both a wide view and zoomed-in details, so you never miss a moment. With advanced package detection and sharp 2K resolution, you'll see exactly who's at your door and what they're carrying.  Enjoy long-lasting battery life and the convenience of a plastic housing, all backed by a 1-year limited warranty.</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1986.9</v>
+        <v>2528</v>
       </c>
       <c r="G40" t="n">
         <v>262</v>
       </c>
       <c r="H40" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -2238,17 +2237,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Capture crystal-clear 1080p HD footage day and night with the Blink Outdoor 4, a limited-edition security camera designed to keep your property safe.  Enjoy up to two years of battery life and peace of mind knowing it's built to withstand the elements. Made from durable plastic, this weather-resistant camera delivers reliable performance wherever you need it. Backed by a one-year limited warranty, the Blink Outdoor 4 is a smart investment in your home's security.</t>
+          <t>Upgrade your home security with the Blink Outdoor 4, a limited-edition security camera delivering crisp 1080p HD video.  This weather-resistant camera boasts a remarkable 2-year battery life, ensuring continuous monitoring without the hassle of frequent charging.  Crafted from durable plastic, the Blink Outdoor 4 is built to withstand the elements and provide reliable protection for your property. Backed by a 1-year limited warranty, you can enjoy peace of mind knowing your investment is protected.</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>838.6</v>
+        <v>1125.4</v>
       </c>
       <c r="G41" t="n">
         <v>262</v>
       </c>
       <c r="H41" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -2282,17 +2281,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Experience unparalleled responsiveness and precision with the Corsair K100 RGB Keyboard. Equipped with Cherry MX Speed keyswitches and boasting a lightning-fast 4000Hz polling rate, every command is executed instantly.  The durable aluminum frame ensures lasting performance, while the spacious layout provides ample room for comfortable and efficient typing.  Backed by a 2-year warranty, the K100 RGB is a premium keyboard built to elevate your gaming and productivity.</t>
+          <t>Experience lightning-fast responsiveness with the Corsair K100 RGB Keyboard.  Crafted with a durable brushed aluminum frame and equipped with Cherry MX Speed switches, this keyboard delivers exceptional performance for both gaming and productivity.  The 4000Hz polling rate ensures ultra-low latency, giving you a competitive edge in every game. Backed by a 2-year warranty, the K100 RGB is a reliable and feature-packed addition to any setup.</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>850.1</v>
+        <v>1698</v>
       </c>
       <c r="G42" t="n">
         <v>264</v>
       </c>
       <c r="H42" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -2326,17 +2325,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>The Logitech MX Master 3S is designed for the ultimate productivity experience.  With its incredibly precise 8K DPI sensor, you'll navigate seamlessly across screens, while the MagSpeed scroll wheel allows for lightning-fast scrolling through documents and web pages.  Connect effortlessly via Bolt or Bluetooth, and choose from a range of stylish colors to match your personal style.  Backed by a 1-year limited warranty, the MX Master 3S is built to last and elevate your workflow.</t>
+          <t>Experience effortless precision with the Logitech MX Master 3S.  Boasting an incredible 8K DPI sensor, this mouse glides smoothly across any surface, ensuring pinpoint accuracy for demanding tasks.  The MagSpeed scroll wheel provides lightning-fast and quiet scrolling, while Bolt and Bluetooth connectivity offer seamless switching between devices.  Choose from a variety of colors to match your style and elevate your productivity with the MX Master 3S. Backed by a 1-year limited warranty, you can trust in its quality and performance.</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>951.2</v>
+        <v>1959.5</v>
       </c>
       <c r="G43" t="n">
         <v>262</v>
       </c>
       <c r="H43" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -2370,17 +2369,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Experience lightning-fast precision and comfort with the Razer DeathAdder V3 Pro. This ultralight gaming mouse weighs a mere 63g, allowing for effortless maneuvers and quick reflexes. Equipped with a 30K DPI Focus Pro sensor, you'll enjoy unparalleled accuracy and tracking, making every click count. The long-lasting battery ensures extended gaming sessions without interruption, while the durable plastic construction guarantees reliable performance. Backed by a 2-year warranty, the DeathAdder V3 Pro is your ultimate weapon for dominating the competition.</t>
+          <t>Dominate your games with the Razer DeathAdder V3 Pro. This ultralight gaming mouse, weighing in at a mere 63 grams,  is engineered for lightning-fast reflexes thanks to its 30K DPI Focus Pro sensor.  Experience unparalleled precision and accuracy, while the long-lasting battery keeps you going through intense gaming marathons. Crafted from durable plastic and backed by a 2-year warranty, the DeathAdder V3 Pro is built to withstand the rigors of competitive play.</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1038.6</v>
+        <v>1153.6</v>
       </c>
       <c r="G44" t="n">
         <v>265</v>
       </c>
       <c r="H44" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -2414,17 +2413,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Experience blazing-fast performance with the Samsung 980 Pro 2TB NVMe SSD. Leveraging the power of PCIe 4.0 technology, this drive delivers incredible read speeds up to 7,000 MB/s, making your applications and files launch in an instant.  Its sleek nickel coating not only enhances aesthetics but also helps dissipate heat for optimal performance. Built with durable PCB and NAND flash material and backed by a 5-year limited warranty, the Samsung 980 Pro ensures reliability and peace of mind for all your storage needs.</t>
+          <t>Experience blazing-fast speeds with the Samsung 980 Pro 2TB NVMe SSD.  Boasting PCIe 4.0 technology and a stunning read speed of up to 7,000 MB/s, this SSD will revolutionize your computing experience.  Crafted with durable PCB and NAND flash material, the 980 Pro features a sleek nickel coating for enhanced heat dissipation. Backed by a 5-year limited warranty, you can trust this SSD to deliver exceptional performance and reliability for years to come.</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1368.8</v>
+        <v>1228.5</v>
       </c>
       <c r="G45" t="n">
         <v>281</v>
       </c>
       <c r="H45" t="n">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -2458,17 +2457,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>The Seagate Portable 5TB HDD is your perfect companion for storing and transporting massive files with ease.  This compact 2.5″ drive boasts a robust 5TB capacity,  allowing you to keep all your important documents, photos, and videos organized and readily accessible.  Simply plug it into any USB 3.0 port for instant plug-and-play functionality.  Encased in a durable plastic shell, this drive is built to withstand the rigors of everyday use, and is backed by a 1-year limited warranty for added peace of mind.</t>
+          <t>Take your files on the go with the Seagate Portable 5TB HDD. This reliable external hard drive boasts a spacious 5TB capacity, perfect for storing photos, videos, and documents. With USB 3.0 connectivity and a plug-and-play design, it's incredibly easy to use. Its compact 2.5-inch form factor makes it lightweight and portable, while the durable plastic shell ensures protection wherever you go. Backed by a 1-year limited warranty, you can trust the Seagate Portable 5TB HDD for all your storage needs.</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>997</v>
+        <v>1330.1</v>
       </c>
       <c r="G46" t="n">
         <v>275</v>
       </c>
       <c r="H46" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -2502,17 +2501,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Capture every epic moment with the SanDisk Extreme PRO 128GB SDXC memory card.  This card boasts blazing-fast UHS-I U3 speeds up to 200MB/s read, ensuring smooth performance for even your most demanding photography and videography.  Built tough with a waterproof design, the Extreme PRO is ready for any adventure. Plus, enjoy peace of mind with SanDisk's lifetime limited warranty, guaranteeing long-lasting reliability for all your precious memories.</t>
+          <t>Capture every moment with confidence using the SanDisk Extreme PRO 128GB SDXC memory card.  This card delivers blazing-fast read speeds of up to 200MB/s, perfect for high-resolution videos and burst photography.  With UHS-I U3 technology, you'll experience smooth performance even in demanding situations.  Built tough with waterproof construction, the Extreme PRO is ready for any adventure. Plus, enjoy peace of mind with SanDisk's lifetime limited warranty.</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>890.1</v>
+        <v>984.5</v>
       </c>
       <c r="G47" t="n">
         <v>271</v>
       </c>
       <c r="H47" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -2546,17 +2545,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Experience lightning-fast performance with the Kingston Fury Beast 32GB DDR5 memory. Boasting a blazing 6000MT/s speed and Intel XMP 3.0 support, this kit unlocks the full potential of your system. The sleek, low-profile aluminum heat spreader ensures optimal cooling while maintaining a stylish aesthetic. Backed by a lifetime warranty, the Kingston Fury Beast 32GB DDR5 is a reliable and energy-efficient upgrade for demanding gamers and professionals alike.</t>
+          <t>Unleash the beast within your PC with the Kingston Fury Beast 32GB DDR5 memory.  This high-performance module boasts an impressive 6000MT/s speed, powered by Intel XMP 3.0 for effortless overclocking. The sleek, low-profile aluminum heatspreader keeps temperatures in check, ensuring optimal energy efficiency. Backed by Kingston's lifetime warranty, the Fury Beast 32GB DDR5 is a reliable and powerful upgrade for any demanding system.</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>890.1</v>
+        <v>1164.6</v>
       </c>
       <c r="G48" t="n">
         <v>273</v>
       </c>
       <c r="H48" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
@@ -2590,17 +2589,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Immerse yourself in the heart-pounding action with the Acer Predator XB273U 27″ Monitor. This large-screen powerhouse boasts a stunning 2560x1440 resolution and a lightning-fast 170Hz refresh rate, delivering ultra-smooth gameplay with vibrant colors thanks to its IPS panel and HDR400 technology. G-Sync Compatible, the XB273U ensures tear-free, stutter-free visuals for an unmatched competitive edge.  Built with a durable plastic and metal stand, this monitor comes backed by a 3-year warranty, giving you peace of mind for years of immersive gaming.</t>
+          <t>Experience next-level gaming with the Acer Predator XB273U 27″ Monitor. This large display boasts a stunning 2560×1440 resolution and a lightning-fast 170Hz refresh rate for ultra-smooth gameplay. The IPS panel delivers vibrant colors and wide viewing angles, while HDR400 enhances contrast and detail for an immersive visual experience. G-Sync Compatible technology ensures tear-free and stutter-free performance. Built with a durable plastic and metal stand, the Predator XB273U is backed by a 3-year warranty, giving you peace of mind for years of epic gaming.</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1151.7</v>
+        <v>1320.9</v>
       </c>
       <c r="G49" t="n">
         <v>283</v>
       </c>
       <c r="H49" t="n">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
@@ -2634,17 +2633,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Immerse yourself in breathtaking clarity with the BenQ PD2725U 27” Monitor. Boasting a stunning 4K UHD IPS display, you'll experience vibrant colors and exceptional detail, thanks to 98% P3 color accuracy.  Seamlessly connect your devices with Thunderbolt 3, ensuring fast data transfer speeds and power delivery. The sleek metal stand provides a sturdy base for your workspace, and with a 3-year warranty, you can enjoy peace of mind knowing your investment is protected.</t>
+          <t>Experience breathtaking visuals with the BenQ PD2725U 27″ Monitor. Its stunning 4K UHD IPS display delivers crystal-clear detail and vibrant colors, covering 98% of the P3 color gamut for exceptional accuracy.  Effortlessly connect your devices with the integrated Thunderbolt 3 port, ensuring fast data transfer speeds and power delivery.  Crafted with a durable metal stand, this monitor is not only beautiful but built to last, backed by a reassuring 3-year warranty.</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>941.3</v>
+        <v>1237.1</v>
       </c>
       <c r="G50" t="n">
         <v>272</v>
       </c>
       <c r="H50" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
@@ -2678,17 +2677,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>The ASUS ProArt PA278QV Monitor is a professional's dream, boasting a stunning 27" 2560x1440 IPS display that covers 100% sRGB for vibrant, accurate colors. Calman Verified ensures exceptional color accuracy, perfect for designers, photographers, and videographers. Its lightweight design and sturdy metal stand make it both portable and reliable, backed by a 3-year warranty for peace of mind.</t>
+          <t>The ASUS ProArt PA278QV Monitor is a dream come true for creatives.  Its vibrant 27" 2560x1440 IPS display covers 100% of the sRGB color gamut, ensuring your work looks stunningly accurate. Calman Verified technology guarantees precise color reproduction, while the light metal stand provides a sleek and stable foundation.  Backed by a 3-year warranty, the PA278QV is an investment in your creative vision.</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>826.5</v>
+        <v>1126.7</v>
       </c>
       <c r="G51" t="n">
         <v>278</v>
       </c>
       <c r="H51" t="n">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>

</xml_diff>